<commit_message>
feat(upload): flag ?reset=1 limpa curva antiga antes do upload
Antes: upload fazia upsert(onConflict=det_id,mes), deixando lixo de meses/
dets que não estão no novo arquivo. Usuário precisava 'limpar' a base
manualmente antes de subir a versão correta.

Agora: quando ?reset=1, o endpoint deleta TODAS as linhas de
planejamento_fisico_det (ou planejamento_fat_direto_det, conforme o tipo
detectado) dos detalhamentos do contrato ANTES de inserir a nova curva.

Frontend sempre passa ?reset=1 no upload — upload é tratado como
'verdade nova', não como merge com a versão anterior. Isso garante que
os totais do contrato e do cronograma convergem exatamente para os
valores da planilha.
</commit_message>
<xml_diff>
--- a/docs/fat direto upload.xlsx
+++ b/docs/fat direto upload.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="99" documentId="11_061FC23109F1F941B261023760305AB482D1CD0D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2CD8399-3C84-4A0E-B819-B6CC2E742A00}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="5760" yWindow="3312" windowWidth="17280" windowHeight="8928" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FÍSICO FINANCEIRO (2)" sheetId="3" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'FÍSICO FINANCEIRO'!$A$1:$M$408</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FÍSICO FINANCEIRO (2)'!$A$2:$K$426</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>

</xml_diff>